<commit_message>
Add Yemen Housing campaign (tracker + excel) + auto-migration for saved data
</commit_message>
<xml_diff>
--- a/site/YetimVakfi_Fundraising_Tracker.xlsx
+++ b/site/YetimVakfi_Fundraising_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Report" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Donations'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Donations'!$A$1:$H$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -860,6 +860,28 @@
         <v/>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="9">
+        <f>IF(Campaigns!A10="","",Campaigns!A10)</f>
+        <v/>
+      </c>
+      <c r="B24" s="10">
+        <f>IF(Campaigns!A10="","",Campaigns!C10)</f>
+        <v/>
+      </c>
+      <c r="C24" s="10">
+        <f>IF(Campaigns!A10="","",Campaigns!D10)</f>
+        <v/>
+      </c>
+      <c r="D24" s="11">
+        <f>IF(Campaigns!A10="","",Campaigns!E10)</f>
+        <v/>
+      </c>
+      <c r="E24" s="10">
+        <f>IF(Campaigns!A10="","",Campaigns!F10)</f>
+        <v/>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -892,7 +914,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D16:D23">
+  <conditionalFormatting sqref="D16:D24">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1218,6 +1240,38 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Yemen Konut Projesi</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Yemen Housing Project</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="D10" s="16">
+        <f>310000+SUMIFS(Donations!G:G,Donations!C:C,A10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="17">
+        <f>IF(C10=0,0,D10/C10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="16">
+        <f>C10-D10</f>
+        <v/>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>5 ev × 42 m² ($36.100) — çadırlardan güvenli evlere</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1226,7 +1280,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E9">
+  <conditionalFormatting sqref="E2:E10">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1250,7 +1304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2177,11 +2231,85 @@
       </c>
       <c r="H25" s="15" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" s="18" t="n">
+        <v>46270</v>
+      </c>
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>Khalid Mansour</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Yemen Konut Projesi</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Sadaka</t>
+        </is>
+      </c>
+      <c r="E26" s="20" t="n">
+        <v>500</v>
+      </c>
+      <c r="F26" s="19" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G26" s="21">
+        <f>IF(F26="USD",E26*Dashboard!B$26,IF(F26="EUR",E26*Dashboard!B$27,E26))</f>
+        <v/>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>Yemen housing</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="n">
+        <v>46252</v>
+      </c>
+      <c r="B27" s="19" t="inlineStr">
+        <is>
+          <t>Sare Demir</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>Yemen Konut Projesi</t>
+        </is>
+      </c>
+      <c r="D27" s="19" t="inlineStr">
+        <is>
+          <t>Tek Seferlik</t>
+        </is>
+      </c>
+      <c r="E27" s="20" t="n">
+        <v>2500</v>
+      </c>
+      <c r="F27" s="19" t="inlineStr">
+        <is>
+          <t>TRY</t>
+        </is>
+      </c>
+      <c r="G27" s="21">
+        <f>IF(F27="USD",E27*Dashboard!B$26,IF(F27="EUR",E27*Dashboard!B$27,E27))</f>
+        <v/>
+      </c>
+      <c r="H27" s="15" t="inlineStr">
+        <is>
+          <t>Sadaka-i cariye</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:H27"/>
   <dataValidations count="3">
     <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Kampanya" error="Listeden bir kampanya seçin." type="list">
-      <formula1>"Yetim Sponsorluğu,Filistin Acil Yardım / Gazze Sıcak Yemek,İyilik Çantası – Kırtasiye,Adak – Akika – Şükür Kurbanı,Zekât &amp; Sadaka Fonu,Yetimhane &amp; Yerleşkeler,Gıda Paketi,Eğitim &amp; Burs Desteği"</formula1>
+      <formula1>"Yetim Sponsorluğu,Filistin Acil Yardım / Gazze Sıcak Yemek,İyilik Çantası – Kırtasiye,Adak – Akika – Şükür Kurbanı,Zekât &amp; Sadaka Fonu,Yetimhane &amp; Yerleşkeler,Gıda Paketi,Eğitim &amp; Burs Desteği,Yemen Konut Projesi"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tek Seferlik,Aylık,Zekât,Sadaka,Fidye,Kurumsal"</formula1>

</xml_diff>

<commit_message>
Remove Yemen campaign/content (tracker + excel + bot) + saved-data cleanup
</commit_message>
<xml_diff>
--- a/site/YetimVakfi_Fundraising_Tracker.xlsx
+++ b/site/YetimVakfi_Fundraising_Tracker.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Report" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Donations'!$A$1:$H$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Donations'!$A$1:$H$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -860,28 +860,6 @@
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="9">
-        <f>IF(Campaigns!A10="","",Campaigns!A10)</f>
-        <v/>
-      </c>
-      <c r="B24" s="10">
-        <f>IF(Campaigns!A10="","",Campaigns!C10)</f>
-        <v/>
-      </c>
-      <c r="C24" s="10">
-        <f>IF(Campaigns!A10="","",Campaigns!D10)</f>
-        <v/>
-      </c>
-      <c r="D24" s="11">
-        <f>IF(Campaigns!A10="","",Campaigns!E10)</f>
-        <v/>
-      </c>
-      <c r="E24" s="10">
-        <f>IF(Campaigns!A10="","",Campaigns!F10)</f>
-        <v/>
-      </c>
-    </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
@@ -914,7 +892,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D16:D24">
+  <conditionalFormatting sqref="D16:D23">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1240,38 +1218,6 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Yemen Konut Projesi</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Yemen Housing Project</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="D10" s="16">
-        <f>310000+SUMIFS(Donations!G:G,Donations!C:C,A10)</f>
-        <v/>
-      </c>
-      <c r="E10" s="17">
-        <f>IF(C10=0,0,D10/C10)</f>
-        <v/>
-      </c>
-      <c r="F10" s="16">
-        <f>C10-D10</f>
-        <v/>
-      </c>
-      <c r="G10" s="15" t="inlineStr">
-        <is>
-          <t>5 ev × 42 m² ($36.100) — çadırlardan güvenli evlere</t>
-        </is>
-      </c>
-    </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -1280,7 +1226,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E2:E10">
+  <conditionalFormatting sqref="E2:E9">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -1304,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2231,85 +2177,11 @@
       </c>
       <c r="H25" s="15" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" s="18" t="n">
-        <v>46270</v>
-      </c>
-      <c r="B26" s="19" t="inlineStr">
-        <is>
-          <t>Khalid Mansour</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Yemen Konut Projesi</t>
-        </is>
-      </c>
-      <c r="D26" s="19" t="inlineStr">
-        <is>
-          <t>Sadaka</t>
-        </is>
-      </c>
-      <c r="E26" s="20" t="n">
-        <v>500</v>
-      </c>
-      <c r="F26" s="19" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G26" s="21">
-        <f>IF(F26="USD",E26*Dashboard!B$26,IF(F26="EUR",E26*Dashboard!B$27,E26))</f>
-        <v/>
-      </c>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>Yemen housing</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="18" t="n">
-        <v>46252</v>
-      </c>
-      <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>Sare Demir</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>Yemen Konut Projesi</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr">
-        <is>
-          <t>Tek Seferlik</t>
-        </is>
-      </c>
-      <c r="E27" s="20" t="n">
-        <v>2500</v>
-      </c>
-      <c r="F27" s="19" t="inlineStr">
-        <is>
-          <t>TRY</t>
-        </is>
-      </c>
-      <c r="G27" s="21">
-        <f>IF(F27="USD",E27*Dashboard!B$26,IF(F27="EUR",E27*Dashboard!B$27,E27))</f>
-        <v/>
-      </c>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t>Sadaka-i cariye</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H27"/>
+  <autoFilter ref="A1:H25"/>
   <dataValidations count="3">
     <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Kampanya" error="Listeden bir kampanya seçin." type="list">
-      <formula1>"Yetim Sponsorluğu,Filistin Acil Yardım / Gazze Sıcak Yemek,İyilik Çantası – Kırtasiye,Adak – Akika – Şükür Kurbanı,Zekât &amp; Sadaka Fonu,Yetimhane &amp; Yerleşkeler,Gıda Paketi,Eğitim &amp; Burs Desteği,Yemen Konut Projesi"</formula1>
+      <formula1>"Yetim Sponsorluğu,Filistin Acil Yardım / Gazze Sıcak Yemek,İyilik Çantası – Kırtasiye,Adak – Akika – Şükür Kurbanı,Zekât &amp; Sadaka Fonu,Yetimhane &amp; Yerleşkeler,Gıda Paketi,Eğitim &amp; Burs Desteği"</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D5000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"Tek Seferlik,Aylık,Zekât,Sadaka,Fidye,Kurumsal"</formula1>

</xml_diff>